<commit_message>
feat(rules): solidify pending vs on-sale tender unit rules in AGENTS.md, scrapers, and update all Excel workbooks & web data
</commit_message>
<xml_diff>
--- a/files/九龙-启德-天玺．天第2期.xlsx
+++ b/files/九龙-启德-天玺．天第2期.xlsx
@@ -26535,7 +26535,7 @@
       </c>
       <c r="F392" s="3" t="inlineStr">
         <is>
-          <t>已定价未售</t>
+          <t>在售</t>
         </is>
       </c>
       <c r="G392" s="3" t="inlineStr">
@@ -29151,7 +29151,7 @@
       </c>
       <c r="F432" s="3" t="inlineStr">
         <is>
-          <t>已定价未售</t>
+          <t>在售</t>
         </is>
       </c>
       <c r="G432" s="3" t="inlineStr">
@@ -43967,12 +43967,12 @@
         </is>
       </c>
       <c r="G22" s="20" t="inlineStr"/>
-      <c r="H22" s="25" t="inlineStr">
+      <c r="H22" s="24" t="inlineStr">
         <is>
           <t>B1 | 478呎 (2房)
 招标单位
 -
-(已定价未售)</t>
+(在售)</t>
         </is>
       </c>
       <c r="I22" s="25" t="inlineStr">
@@ -44347,12 +44347,12 @@
         </is>
       </c>
       <c r="G26" s="20" t="inlineStr"/>
-      <c r="H26" s="25" t="inlineStr">
+      <c r="H26" s="24" t="inlineStr">
         <is>
           <t>B1 | 478呎 (2房)
 招标单位
 -
-(已定价未售)</t>
+(在售)</t>
         </is>
       </c>
       <c r="I26" s="25" t="inlineStr">

</xml_diff>